<commit_message>
Add instruction for SQL-query construction.
</commit_message>
<xml_diff>
--- a/Sensors_Description/climate_control_theorist_schema.xlsx
+++ b/Sensors_Description/climate_control_theorist_schema.xlsx
@@ -15129,7 +15129,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
         <v>33</v>
       </c>
@@ -16905,7 +16905,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
         <v>33</v>
       </c>
@@ -18681,7 +18681,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
         <v>33</v>
       </c>
@@ -20457,7 +20457,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
         <v>33</v>
       </c>
@@ -20568,7 +20568,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
         <v>33</v>
       </c>
@@ -20679,7 +20679,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
         <v>33</v>
       </c>
@@ -25785,7 +25785,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="6" t="s">
         <v>33</v>
       </c>
@@ -25896,7 +25896,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="6" t="s">
         <v>33</v>
       </c>
@@ -26007,7 +26007,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="6" t="s">
         <v>33</v>
       </c>
@@ -27117,7 +27117,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="6" t="s">
         <v>33</v>
       </c>
@@ -27228,7 +27228,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="6" t="s">
         <v>33</v>
       </c>
@@ -27339,7 +27339,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="72" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="6" t="s">
         <v>33</v>
       </c>
@@ -42150,9 +42150,19 @@
     </row>
   </sheetData>
   <autoFilter ref="A3:AK248">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Carbon dioxide concentration"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="2">
       <filters>
         <filter val="C_CO2,basalt"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="6">
+      <filters>
+        <filter val="LEO West"/>
       </filters>
     </filterColumn>
     <filterColumn colId="20">
@@ -42162,7 +42172,7 @@
     </filterColumn>
     <filterColumn colId="21">
       <filters>
-        <filter val="4"/>
+        <filter val="10"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>